<commit_message>
Master data added on 27th May, 2024 -2
</commit_message>
<xml_diff>
--- a/MasterDataReader-Project/XlsxReader2/src/main/java/com/pwc/xlsx/27-05-2024 MASTER DATA.xlsx
+++ b/MasterDataReader-Project/XlsxReader2/src/main/java/com/pwc/xlsx/27-05-2024 MASTER DATA.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stpr918\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stpr918\Documents\OBPAS\Mater data folder\Master data 2024\May 2024\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{505E57A4-E274-43F8-ADE7-D1E12DB20961}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40D1ECE4-B017-4872-91DE-57F0559A7920}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="83">
   <si>
     <t>S.no.</t>
   </si>
@@ -242,6 +242,36 @@
   </si>
   <si>
     <t>3, 3/1</t>
+  </si>
+  <si>
+    <t>High Rise Building</t>
+  </si>
+  <si>
+    <t>A-H</t>
+  </si>
+  <si>
+    <t>47A</t>
+  </si>
+  <si>
+    <t>A6</t>
+  </si>
+  <si>
+    <t>8C</t>
+  </si>
+  <si>
+    <t>ONE_KANAL</t>
+  </si>
+  <si>
+    <t>60F</t>
+  </si>
+  <si>
+    <t>75F</t>
+  </si>
+  <si>
+    <t>35F</t>
+  </si>
+  <si>
+    <t>25F6</t>
   </si>
 </sst>
 </file>
@@ -319,7 +349,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -368,6 +398,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -683,7 +716,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W12"/>
+  <dimension ref="A1:W15"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="4"/>
@@ -1553,6 +1586,219 @@
         <v>42</v>
       </c>
     </row>
+    <row r="13" spans="1:23" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="10">
+        <v>12</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="E13" s="5">
+        <v>1</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="J13" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="L13" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="M13" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="N13" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="O13" s="5">
+        <v>3</v>
+      </c>
+      <c r="P13" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q13" s="5">
+        <v>2</v>
+      </c>
+      <c r="R13" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="S13" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="T13" s="5">
+        <v>0</v>
+      </c>
+      <c r="U13" s="5">
+        <v>0</v>
+      </c>
+      <c r="V13" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="W13" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A14" s="5">
+        <v>13</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E14" s="5">
+        <v>1</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="G14" s="5">
+        <v>1128</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J14" s="6">
+        <v>418.06</v>
+      </c>
+      <c r="K14" s="6">
+        <v>499.99</v>
+      </c>
+      <c r="L14" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="M14" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="N14" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="O14" s="6">
+        <v>3</v>
+      </c>
+      <c r="P14" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q14" s="18">
+        <v>1.5000100000000001</v>
+      </c>
+      <c r="R14" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="S14" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="T14" s="5">
+        <v>0</v>
+      </c>
+      <c r="U14" s="5">
+        <v>0</v>
+      </c>
+      <c r="V14" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="W14" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A15" s="5">
+        <v>13</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E15" s="5">
+        <v>1</v>
+      </c>
+      <c r="F15" s="5">
+        <v>5</v>
+      </c>
+      <c r="G15" s="5">
+        <v>22</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="K15" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L15" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="M15" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N15" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="O15" s="6">
+        <v>2</v>
+      </c>
+      <c r="P15" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="Q15" s="18">
+        <v>1</v>
+      </c>
+      <c r="R15" s="5">
+        <v>50</v>
+      </c>
+      <c r="S15" s="5">
+        <v>0</v>
+      </c>
+      <c r="T15" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="U15" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="V15" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="W15" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:W1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>